<commit_message>
Added --ELTM output variable.  Positive test case 1 is showing an error.
</commit_message>
<xml_diff>
--- a/rules/CORE-000142/negative/01/data/unit-test-coreid-CG0241-negative 1.xlsx
+++ b/rules/CORE-000142/negative/01/data/unit-test-coreid-CG0241-negative 1.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -49,6 +49,10 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
@@ -73,7 +77,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -93,6 +97,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -128,16 +138,17 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -480,10 +491,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -507,10 +518,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="B2" s="2" t="str">
+      <c r="A2" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="B2" s="4" t="str">
         <v>Functional Tests</v>
       </c>
     </row>
@@ -523,7 +534,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F25"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -546,42 +557,42 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C2" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D2" s="2">
+      <c r="B2" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C2" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D2" s="4">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="4" t="str">
         <v>FTTPT</v>
       </c>
-      <c r="F2" s="2" t="str">
+      <c r="F2" s="4" t="str">
         <v>30 MIN POST</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C3" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D3" s="2">
+      <c r="B3" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C3" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D3" s="4">
         <v>5</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E3" s="4" t="str">
         <v>FTTPTNUM</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="4">
         <v>1</v>
       </c>
     </row>
@@ -599,110 +610,110 @@
         <v>5</v>
       </c>
       <c r="E4" s="2" t="str">
+        <v>FTTPTREF</v>
+      </c>
+      <c r="F4" s="2" t="str">
+        <v>DOSE</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C5" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D5" s="4">
+        <v>5</v>
+      </c>
+      <c r="E5" s="4" t="str">
         <v>FTELTM</v>
       </c>
-      <c r="F4" s="2" t="str">
+      <c r="F5" s="4" t="str">
         <v>PT30M</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2">
+    <row r="6">
+      <c r="A6" s="4">
         <v>1</v>
       </c>
-      <c r="B5" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C5" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D5" s="2">
+      <c r="B6" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C6" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D6" s="4">
         <v>5</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E6" s="4" t="str">
         <v>VISITNUM</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F6" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2">
+    <row r="7">
+      <c r="A7" s="4">
         <v>1</v>
       </c>
-      <c r="B6" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C6" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D6" s="2">
+      <c r="B7" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C7" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D7" s="4">
         <v>5</v>
       </c>
-      <c r="E6" s="2" t="str">
+      <c r="E7" s="4" t="str">
         <v>DOMAIN</v>
       </c>
-      <c r="F6" s="2" t="str">
+      <c r="F7" s="4" t="str">
         <v>FT</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2">
+    <row r="8">
+      <c r="A8" s="4">
         <v>2</v>
       </c>
-      <c r="B7" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C7" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D7" s="2">
+      <c r="B8" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C8" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D8" s="4">
         <v>6</v>
       </c>
-      <c r="E7" s="2" t="str">
+      <c r="E8" s="4" t="str">
         <v>FTTPT</v>
       </c>
-      <c r="F7" s="2" t="str">
+      <c r="F8" s="4" t="str">
         <v>30 MIN POST</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2">
+    <row r="9">
+      <c r="A9" s="4">
         <v>2</v>
       </c>
-      <c r="B8" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C8" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D8" s="2">
+      <c r="B9" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C9" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D9" s="4">
         <v>6</v>
       </c>
-      <c r="E8" s="2" t="str">
+      <c r="E9" s="4" t="str">
         <v>FTTPTNUM</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F9" s="4">
         <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2">
-        <v>2</v>
-      </c>
-      <c r="B9" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C9" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D9" s="2">
-        <v>6</v>
-      </c>
-      <c r="E9" s="2" t="str">
-        <v>FTELTM</v>
-      </c>
-      <c r="F9" s="2" t="str">
-        <v>PT03M</v>
       </c>
     </row>
     <row r="10">
@@ -719,110 +730,110 @@
         <v>6</v>
       </c>
       <c r="E10" s="2" t="str">
+        <v>FTTPTREF</v>
+      </c>
+      <c r="F10" s="2" t="str">
+        <v>DOSE</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4">
+        <v>2</v>
+      </c>
+      <c r="B11" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C11" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D11" s="4">
+        <v>6</v>
+      </c>
+      <c r="E11" s="4" t="str">
+        <v>FTELTM</v>
+      </c>
+      <c r="F11" s="4" t="str">
+        <v>PT03M</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4">
+        <v>2</v>
+      </c>
+      <c r="B12" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C12" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D12" s="4">
+        <v>6</v>
+      </c>
+      <c r="E12" s="4" t="str">
         <v>VISITNUM</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F12" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2">
+    <row r="13">
+      <c r="A13" s="4">
         <v>2</v>
       </c>
-      <c r="B11" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C11" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D11" s="2">
+      <c r="B13" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C13" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D13" s="4">
         <v>6</v>
       </c>
-      <c r="E11" s="2" t="str">
+      <c r="E13" s="4" t="str">
         <v>DOMAIN</v>
       </c>
-      <c r="F11" s="2" t="str">
+      <c r="F13" s="4" t="str">
         <v>FT</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2">
+    <row r="14">
+      <c r="A14" s="4">
         <v>3</v>
       </c>
-      <c r="B12" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C12" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D12" s="2">
+      <c r="B14" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C14" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D14" s="4">
         <v>7</v>
       </c>
-      <c r="E12" s="2" t="str">
+      <c r="E14" s="4" t="str">
         <v>FTTPT</v>
       </c>
-      <c r="F12" s="2" t="str">
+      <c r="F14" s="4" t="str">
         <v>90 MIN POST</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2">
+    <row r="15">
+      <c r="A15" s="4">
         <v>3</v>
       </c>
-      <c r="B13" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C13" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D13" s="2">
+      <c r="B15" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C15" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D15" s="4">
         <v>7</v>
       </c>
-      <c r="E13" s="2" t="str">
+      <c r="E15" s="4" t="str">
         <v>FTTPTNUM</v>
       </c>
-      <c r="F13" s="2">
+      <c r="F15" s="4">
         <v>2</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2">
-        <v>3</v>
-      </c>
-      <c r="B14" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C14" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D14" s="2">
-        <v>7</v>
-      </c>
-      <c r="E14" s="2" t="str">
-        <v>FTELTM</v>
-      </c>
-      <c r="F14" s="2" t="str">
-        <v>PT1H</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2">
-        <v>3</v>
-      </c>
-      <c r="B15" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C15" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D15" s="2">
-        <v>7</v>
-      </c>
-      <c r="E15" s="2" t="str">
-        <v>VISITNUM</v>
-      </c>
-      <c r="F15" s="2">
-        <v>201</v>
       </c>
     </row>
     <row r="16">
@@ -839,115 +850,195 @@
         <v>7</v>
       </c>
       <c r="E16" s="2" t="str">
+        <v>FTTPTREF</v>
+      </c>
+      <c r="F16" s="2" t="str">
+        <v>BREAKFAST</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4">
+        <v>3</v>
+      </c>
+      <c r="B17" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C17" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D17" s="4">
+        <v>7</v>
+      </c>
+      <c r="E17" s="4" t="str">
+        <v>FTELTM</v>
+      </c>
+      <c r="F17" s="4" t="str">
+        <v>PT1H</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4">
+        <v>3</v>
+      </c>
+      <c r="B18" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C18" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D18" s="4">
+        <v>7</v>
+      </c>
+      <c r="E18" s="4" t="str">
+        <v>VISITNUM</v>
+      </c>
+      <c r="F18" s="4">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4">
+        <v>3</v>
+      </c>
+      <c r="B19" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C19" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D19" s="4">
+        <v>7</v>
+      </c>
+      <c r="E19" s="4" t="str">
         <v>DOMAIN</v>
       </c>
-      <c r="F16" s="2" t="str">
+      <c r="F19" s="4" t="str">
         <v>FT</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2">
+    <row r="20">
+      <c r="A20" s="4">
         <v>4</v>
       </c>
-      <c r="B17" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C17" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D17" s="2">
+      <c r="B20" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C20" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D20" s="4">
         <v>8</v>
       </c>
-      <c r="E17" s="2" t="str">
+      <c r="E20" s="4" t="str">
         <v>FTTPT</v>
       </c>
-      <c r="F17" s="2" t="str">
+      <c r="F20" s="4" t="str">
         <v>90 MIN POST</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2">
+    <row r="21">
+      <c r="A21" s="4">
         <v>4</v>
       </c>
-      <c r="B18" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C18" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D18" s="2">
+      <c r="B21" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C21" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D21" s="4">
         <v>8</v>
       </c>
-      <c r="E18" s="2" t="str">
+      <c r="E21" s="4" t="str">
         <v>FTTPTNUM</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F21" s="4">
         <v>2</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2">
+    <row r="22">
+      <c r="A22" s="2">
         <v>4</v>
       </c>
-      <c r="B19" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C19" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D19" s="2">
+      <c r="B22" s="2" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C22" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D22" s="2">
         <v>8</v>
       </c>
-      <c r="E19" s="2" t="str">
+      <c r="E22" s="2" t="str">
+        <v>FTTPTREF</v>
+      </c>
+      <c r="F22" s="2" t="str">
+        <v>BREAKFAST</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4">
+        <v>4</v>
+      </c>
+      <c r="B23" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C23" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D23" s="4">
+        <v>8</v>
+      </c>
+      <c r="E23" s="4" t="str">
         <v>FTELTM</v>
       </c>
-      <c r="F19" s="2" t="str">
+      <c r="F23" s="4" t="str">
         <v>PT2H</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2">
+    <row r="24">
+      <c r="A24" s="4">
         <v>4</v>
       </c>
-      <c r="B20" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C20" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D20" s="2">
+      <c r="B24" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C24" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D24" s="4">
         <v>8</v>
       </c>
-      <c r="E20" s="2" t="str">
+      <c r="E24" s="4" t="str">
         <v>VISITNUM</v>
       </c>
-      <c r="F20" s="2">
+      <c r="F24" s="4">
         <v>201</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2">
+    <row r="25">
+      <c r="A25" s="4">
         <v>4</v>
       </c>
-      <c r="B21" s="2" t="str">
-        <v>ft.xpt</v>
-      </c>
-      <c r="C21" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D21" s="2">
+      <c r="B25" s="4" t="str">
+        <v>ft.xpt</v>
+      </c>
+      <c r="C25" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D25" s="4">
         <v>8</v>
       </c>
-      <c r="E21" s="2" t="str">
+      <c r="E25" s="4" t="str">
         <v>DOMAIN</v>
       </c>
-      <c r="F21" s="2" t="str">
+      <c r="F25" s="4" t="str">
         <v>FT</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F25"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1025,262 +1116,262 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="4" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="4" t="str">
+      <c r="D2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="4" t="str">
+      <c r="E2" s="5" t="str">
         <v>Short Name of Test</v>
       </c>
-      <c r="F2" s="4" t="str">
+      <c r="F2" s="5" t="str">
         <v>Name of Test</v>
       </c>
-      <c r="G2" s="4" t="str">
+      <c r="G2" s="5" t="str">
         <v>Category</v>
       </c>
-      <c r="H2" s="4" t="str">
+      <c r="H2" s="5" t="str">
         <v>Subcategory</v>
       </c>
-      <c r="I2" s="4" t="str">
+      <c r="I2" s="6" t="str">
         <v>Result or Finding in Original Units</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Result or Finding in Standard Format</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="6" t="str">
         <v>Numeric Result/Finding in Standard Units</v>
       </c>
-      <c r="L2" s="5" t="str">
+      <c r="L2" s="6" t="str">
         <v>Last Observation Before Exposure Flag</v>
       </c>
-      <c r="M2" s="5" t="str">
+      <c r="M2" s="6" t="str">
         <v>Repetition Number</v>
       </c>
-      <c r="N2" s="5" t="str">
+      <c r="N2" s="6" t="str">
         <v>Visit Number</v>
       </c>
-      <c r="O2" s="5" t="str">
+      <c r="O2" s="6" t="str">
         <v>Visit Name</v>
       </c>
-      <c r="P2" s="5" t="str">
+      <c r="P2" s="6" t="str">
         <v>Epoch</v>
       </c>
-      <c r="Q2" s="5" t="str">
+      <c r="Q2" s="6" t="str">
         <v>Date/Time of Test</v>
       </c>
-      <c r="R2" s="5" t="str">
+      <c r="R2" s="6" t="str">
         <v>Study Day of Test</v>
       </c>
-      <c r="S2" s="5" t="str">
+      <c r="S2" s="6" t="str">
         <v>Planned Time Point Name</v>
       </c>
-      <c r="T2" s="5" t="str">
+      <c r="T2" s="6" t="str">
         <v>Planned Time Point Number</v>
       </c>
-      <c r="U2" s="5" t="str">
+      <c r="U2" s="6" t="str">
         <v>Planned Elapsed Time from Time Point Ref</v>
       </c>
-      <c r="V2" s="5" t="str">
+      <c r="V2" s="6" t="str">
         <v>Time Point Reference</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
+      <c r="A3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="B3" s="5" t="str">
+      <c r="B3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="C3" s="5" t="str">
+      <c r="C3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="D3" s="5" t="str">
+      <c r="D3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="5" t="str">
+      <c r="E3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="F3" s="5" t="str">
+      <c r="F3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="G3" s="5" t="str">
+      <c r="G3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="H3" s="5" t="str">
+      <c r="H3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="I3" s="5" t="str">
+      <c r="I3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="J3" s="5" t="str">
+      <c r="J3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="K3" s="5" t="str">
+      <c r="K3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="L3" s="5" t="str">
+      <c r="L3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="M3" s="5" t="str">
+      <c r="M3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="N3" s="5" t="str">
+      <c r="N3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="O3" s="5" t="str">
+      <c r="O3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="P3" s="5" t="str">
+      <c r="P3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="Q3" s="5" t="str">
+      <c r="Q3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="R3" s="5" t="str">
+      <c r="R3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="S3" s="5" t="str">
+      <c r="S3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="T3" s="5" t="str">
+      <c r="T3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="U3" s="5" t="str">
+      <c r="U3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="V3" s="5" t="str">
+      <c r="V3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>12</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>8</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="6">
         <v>8</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="6">
         <v>7</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="6">
         <v>23</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="6">
         <v>8</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="6">
         <v>200</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="6">
         <v>12</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="6">
         <v>200</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="6">
         <v>8</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="6">
         <v>1</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="6">
         <v>8</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="6">
         <v>8</v>
       </c>
-      <c r="O4" s="5">
+      <c r="O4" s="6">
         <v>200</v>
       </c>
-      <c r="P4" s="5">
+      <c r="P4" s="6">
         <v>9</v>
       </c>
-      <c r="Q4" s="5">
+      <c r="Q4" s="6">
         <v>19</v>
       </c>
-      <c r="R4" s="5">
+      <c r="R4" s="6">
         <v>8</v>
       </c>
-      <c r="S4" s="5">
+      <c r="S4" s="6">
         <v>200</v>
       </c>
-      <c r="T4" s="5">
+      <c r="T4" s="6">
         <v>8</v>
       </c>
-      <c r="U4" s="5">
+      <c r="U4" s="6">
         <v>200</v>
       </c>
-      <c r="V4" s="5">
+      <c r="V4" s="6">
         <v>200</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="str">
+      <c r="A5" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
       <c r="B5" s="7" t="str">
         <v>FT</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="4">
         <v>120</v>
       </c>
-      <c r="E5" s="6" t="str">
+      <c r="E5" s="4" t="str">
         <v>AVL0201</v>
       </c>
-      <c r="F5" s="6" t="str">
+      <c r="F5" s="4" t="str">
         <v>AVL02-List A Word 1</v>
       </c>
-      <c r="G5" s="6" t="str">
+      <c r="G5" s="4" t="str">
         <v>AVLT-REY</v>
       </c>
-      <c r="H5" s="6" t="str">
+      <c r="H5" s="4" t="str">
         <v>FORM 1</v>
       </c>
-      <c r="I5" s="6" t="str">
+      <c r="I5" s="4" t="str">
         <v>RECALLED</v>
       </c>
-      <c r="J5" s="6" t="str">
+      <c r="J5" s="4" t="str">
         <v>RECALLED</v>
       </c>
-      <c r="K5" s="2" t="str">
+      <c r="K5" s="4" t="str">
         <v/>
       </c>
-      <c r="L5" s="6" t="str">
+      <c r="L5" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="M5" s="6">
+      <c r="M5" s="4">
         <v>7</v>
       </c>
       <c r="N5" s="7">
         <v>2</v>
       </c>
-      <c r="O5" s="6" t="str">
+      <c r="O5" s="4" t="str">
         <v>SCREENING 2</v>
       </c>
-      <c r="P5" s="6" t="str">
+      <c r="P5" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="Q5" s="6" t="str">
+      <c r="Q5" s="4" t="str">
         <v>2012-11-28T13:00</v>
       </c>
-      <c r="R5" s="6">
+      <c r="R5" s="4">
         <v>-2</v>
       </c>
       <c r="S5" s="7" t="str">
@@ -1292,131 +1383,131 @@
       <c r="U5" s="7" t="str">
         <v>PT30M</v>
       </c>
-      <c r="V5" s="6" t="str">
+      <c r="V5" s="7" t="str">
         <v>DOSE</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="str">
+      <c r="A6" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
       <c r="B6" s="7" t="str">
         <v>FT</v>
       </c>
-      <c r="C6" s="6" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <v>121</v>
       </c>
-      <c r="E6" s="6" t="str">
+      <c r="E6" s="4" t="str">
         <v>AVL0202</v>
       </c>
-      <c r="F6" s="6" t="str">
+      <c r="F6" s="4" t="str">
         <v>AVL02-List A Word 2</v>
       </c>
-      <c r="G6" s="6" t="str">
+      <c r="G6" s="4" t="str">
         <v>AVLT-REY</v>
       </c>
-      <c r="H6" s="6" t="str">
+      <c r="H6" s="4" t="str">
         <v>FORM 1</v>
       </c>
-      <c r="I6" s="6" t="str">
+      <c r="I6" s="4" t="str">
         <v>RECALLED</v>
       </c>
-      <c r="J6" s="6" t="str">
+      <c r="J6" s="4" t="str">
         <v>RECALLED</v>
       </c>
-      <c r="K6" s="2" t="str">
+      <c r="K6" s="4" t="str">
         <v/>
       </c>
-      <c r="L6" s="6" t="str">
+      <c r="L6" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="M6" s="6">
+      <c r="M6" s="4">
         <v>7</v>
       </c>
       <c r="N6" s="7">
         <v>2</v>
       </c>
-      <c r="O6" s="6" t="str">
+      <c r="O6" s="4" t="str">
         <v>SCREENING 2</v>
       </c>
-      <c r="P6" s="6" t="str">
+      <c r="P6" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="Q6" s="6" t="str">
+      <c r="Q6" s="4" t="str">
         <v>2012-11-28T13:00</v>
       </c>
-      <c r="R6" s="6">
+      <c r="R6" s="4">
         <v>-2</v>
       </c>
       <c r="S6" s="7" t="str">
         <v>30 MIN POST</v>
       </c>
-      <c r="T6" s="7" t="str">
+      <c r="T6" s="8" t="str">
         <v>1</v>
       </c>
       <c r="U6" s="8" t="str">
         <v>PT03M</v>
       </c>
-      <c r="V6" s="6" t="str">
+      <c r="V6" s="9" t="str">
         <v>DOSE</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="str">
+      <c r="A7" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
       <c r="B7" s="8" t="str">
         <v>FT</v>
       </c>
-      <c r="C7" s="6" t="str">
+      <c r="C7" s="4" t="str">
         <v>CDISC007</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="4">
         <v>134</v>
       </c>
-      <c r="E7" s="6" t="str">
+      <c r="E7" s="4" t="str">
         <v>AVL0215</v>
       </c>
-      <c r="F7" s="6" t="str">
+      <c r="F7" s="4" t="str">
         <v>AVL02-List A Word 15</v>
       </c>
-      <c r="G7" s="6" t="str">
+      <c r="G7" s="4" t="str">
         <v>AVLT-REY</v>
       </c>
-      <c r="H7" s="6" t="str">
+      <c r="H7" s="4" t="str">
         <v>FORM 1</v>
       </c>
-      <c r="I7" s="6" t="str">
+      <c r="I7" s="4" t="str">
         <v>RECALLED</v>
       </c>
-      <c r="J7" s="6" t="str">
+      <c r="J7" s="4" t="str">
         <v>RECALLED</v>
       </c>
-      <c r="K7" s="2" t="str">
+      <c r="K7" s="4" t="str">
         <v/>
       </c>
-      <c r="L7" s="2" t="str">
+      <c r="L7" s="4" t="str">
         <v/>
       </c>
-      <c r="M7" s="6">
+      <c r="M7" s="4">
         <v>7</v>
       </c>
       <c r="N7" s="8" t="str">
         <v>201</v>
       </c>
-      <c r="O7" s="6" t="str">
+      <c r="O7" s="4" t="str">
         <v>EARLY DISCONTINUATION RETRIEVAL</v>
       </c>
-      <c r="P7" s="6" t="str">
+      <c r="P7" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="Q7" s="6" t="str">
+      <c r="Q7" s="4" t="str">
         <v>2013-06-20T10:00</v>
       </c>
-      <c r="R7" s="6">
+      <c r="R7" s="4">
         <v>167</v>
       </c>
       <c r="S7" s="8" t="str">
@@ -1428,63 +1519,63 @@
       <c r="U7" s="8" t="str">
         <v>PT1H</v>
       </c>
-      <c r="V7" s="6" t="str">
+      <c r="V7" s="7" t="str">
         <v>BREAKFAST</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="str">
+      <c r="A8" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
       <c r="B8" s="8" t="str">
         <v>FT</v>
       </c>
-      <c r="C8" s="6" t="str">
+      <c r="C8" s="4" t="str">
         <v>CDISC007</v>
       </c>
-      <c r="D8" s="6" t="str">
+      <c r="D8" s="4" t="str">
         <v>135</v>
       </c>
-      <c r="E8" s="6" t="str">
+      <c r="E8" s="4" t="str">
         <v>AVL0216</v>
       </c>
-      <c r="F8" s="6" t="str">
+      <c r="F8" s="4" t="str">
         <v>AVL02-List A Word 16</v>
       </c>
-      <c r="G8" s="6" t="str">
+      <c r="G8" s="4" t="str">
         <v>AVLT-REY</v>
       </c>
-      <c r="H8" s="6" t="str">
+      <c r="H8" s="4" t="str">
         <v>FORM 1</v>
       </c>
-      <c r="I8" s="6" t="str">
+      <c r="I8" s="4" t="str">
         <v>RECALLED</v>
       </c>
-      <c r="J8" s="6" t="str">
+      <c r="J8" s="4" t="str">
         <v>RECALLED</v>
       </c>
-      <c r="K8" s="6" t="str">
+      <c r="K8" s="4" t="str">
         <v/>
       </c>
-      <c r="L8" s="6" t="str">
+      <c r="L8" s="4" t="str">
         <v/>
       </c>
-      <c r="M8" s="6">
+      <c r="M8" s="4">
         <v>7</v>
       </c>
       <c r="N8" s="8" t="str">
         <v>201</v>
       </c>
-      <c r="O8" s="6" t="str">
+      <c r="O8" s="4" t="str">
         <v>EARLY DISCONTINUATION RETRIEVAL</v>
       </c>
-      <c r="P8" s="6" t="str">
+      <c r="P8" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="Q8" s="6" t="str">
+      <c r="Q8" s="4" t="str">
         <v>2013-06-20T10:00</v>
       </c>
-      <c r="R8" s="6">
+      <c r="R8" s="4">
         <v>167</v>
       </c>
       <c r="S8" s="8" t="str">
@@ -1496,7 +1587,7 @@
       <c r="U8" s="8" t="str">
         <v>PT2H</v>
       </c>
-      <c r="V8" s="6" t="str">
+      <c r="V8" s="7" t="str">
         <v>BREAKFAST</v>
       </c>
     </row>

</xml_diff>